<commit_message>
feat: replace concurrent ribbon with period regimes on the main spine
</commit_message>
<xml_diff>
--- a/archive/china_history_v9.xlsx
+++ b/archive/china_history_v9.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K78"/>
+  <dimension ref="A1:K81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3353,7 +3353,7 @@
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>south</t>
+          <t>main</t>
         </is>
       </c>
       <c r="J69" t="n">
@@ -3752,6 +3752,114 @@
       <c r="K78" t="inlineStr">
         <is>
           <t>Manchu dynasty ruling a multiethnic empire</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>R_3K</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>regime</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>Three Kingdoms</t>
+        </is>
+      </c>
+      <c r="E79" t="n">
+        <v>220</v>
+      </c>
+      <c r="F79" t="n">
+        <v>280</v>
+      </c>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="J79" t="n">
+        <v>3</v>
+      </c>
+      <c r="K79" t="inlineStr">
+        <is>
+          <t>Period of three rival kingdoms after Han collapse, ending with Western Jin's reunification</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>R_NSD</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>regime</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>Northern and Southern Dynasties</t>
+        </is>
+      </c>
+      <c r="E80" t="n">
+        <v>420</v>
+      </c>
+      <c r="F80" t="n">
+        <v>589</v>
+      </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="J80" t="n">
+        <v>3</v>
+      </c>
+      <c r="K80" t="inlineStr">
+        <is>
+          <t>Period of fragmented north-south rule between Western Jin's fall and Sui reunification</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>R_5D10K</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>regime</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>Five Dynasties and Ten Kingdoms</t>
+        </is>
+      </c>
+      <c r="E81" t="n">
+        <v>907</v>
+      </c>
+      <c r="F81" t="n">
+        <v>960</v>
+      </c>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="J81" t="n">
+        <v>2</v>
+      </c>
+      <c r="K81" t="inlineStr">
+        <is>
+          <t>Brief turbulent interregnum between Tang's collapse and Northern Song's reunification</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: merge Western Jin into Jin (280-420) and place PRC callout below the snake
</commit_message>
<xml_diff>
--- a/archive/china_history_v9.xlsx
+++ b/archive/china_history_v9.xlsx
@@ -1802,14 +1802,14 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Western Jin</t>
+          <t>Jin</t>
         </is>
       </c>
       <c r="E33" t="n">
-        <v>266</v>
+        <v>280</v>
       </c>
       <c r="F33" t="n">
-        <v>316</v>
+        <v>420</v>
       </c>
       <c r="I33" t="inlineStr">
         <is>
@@ -1821,7 +1821,7 @@
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>Short reunification</t>
+          <t>Reunified rule under the Sima clan after Three Kingdoms, fragmenting into Eastern Jin after losing the north</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: side-mode callout for Xin and close Xin-to-Eastern-Han gap
</commit_message>
<xml_diff>
--- a/archive/china_history_v9.xlsx
+++ b/archive/china_history_v9.xlsx
@@ -1257,7 +1257,7 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="F20" t="n">
         <v>220</v>
@@ -1272,7 +1272,7 @@
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>Restoration</t>
+          <t>Restored Han rule under Liu Xiu after Wang Mang Xin collapse, including the Gengshi interregnum</t>
         </is>
       </c>
     </row>

</xml_diff>